<commit_message>
Adding notes on portability. Fixing table of contents.
</commit_message>
<xml_diff>
--- a/Machine Learning/MLOps/AI Studios/images/Comparison.xlsx
+++ b/Machine Learning/MLOps/AI Studios/images/Comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\taylor.schneider\git\ml-training-jupyter-notebooks\Machine Learning\MLOps\AI Studios\images\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A859CA7-4187-43DC-9F7B-39EDD70958A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{329B7B86-29FA-4E7C-AAE6-87357BFC94C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F72EB834-3690-4F9E-98AA-05EACDBE3276}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="55">
   <si>
     <t>Solution / Feature</t>
   </si>
@@ -199,6 +199,12 @@
   </si>
   <si>
     <t>Both</t>
+  </si>
+  <si>
+    <t>Portable</t>
+  </si>
+  <si>
+    <t>* UI Only, No SDK</t>
   </si>
 </sst>
 </file>
@@ -328,9 +334,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -368,7 +374,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -474,7 +480,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -616,7 +622,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -624,7 +630,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B1923B-0AEE-4BE7-89E9-C5B9C04C759A}">
-  <dimension ref="A1:Y18"/>
+  <dimension ref="A1:Z18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
@@ -632,18 +638,18 @@
     <col min="4" max="4" width="6.33203125" style="1" customWidth="1"/>
     <col min="5" max="7" width="5.5546875" style="1" customWidth="1"/>
     <col min="8" max="8" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.77734375" style="1" customWidth="1"/>
     <col min="11" max="11" width="8.77734375" style="1" customWidth="1"/>
     <col min="12" max="12" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6.5546875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="5.88671875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="5.109375" style="1" customWidth="1"/>
-    <col min="16" max="16" width="22.109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="14" max="15" width="5.88671875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="5.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="22.109375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="6" t="s">
         <v>0</v>
@@ -685,15 +691,17 @@
         <v>30</v>
       </c>
       <c r="O1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="Q1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="R1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="R1" s="2"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
       <c r="U1" s="2"/>
@@ -701,8 +709,9 @@
       <c r="W1" s="2"/>
       <c r="X1" s="2"/>
       <c r="Y1" s="2"/>
-    </row>
-    <row r="2" spans="1:25" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="Z1" s="2"/>
+    </row>
+    <row r="2" spans="1:26" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="10" t="s">
         <v>5</v>
@@ -744,15 +753,17 @@
         <v>15</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="P2" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q2" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="Q2" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="R2" s="2"/>
+      <c r="R2" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
@@ -760,8 +771,9 @@
       <c r="W2" s="2"/>
       <c r="X2" s="2"/>
       <c r="Y2" s="2"/>
-    </row>
-    <row r="3" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="Z2" s="2"/>
+    </row>
+    <row r="3" spans="1:26" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="10" t="s">
         <v>19</v>
@@ -803,15 +815,17 @@
         <v>15</v>
       </c>
       <c r="O3" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="P3" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q3" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="R3" s="2"/>
+      <c r="R3" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
@@ -819,8 +833,9 @@
       <c r="W3" s="2"/>
       <c r="X3" s="2"/>
       <c r="Y3" s="2"/>
-    </row>
-    <row r="4" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="Z3" s="2"/>
+    </row>
+    <row r="4" spans="1:26" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="10" t="s">
         <v>6</v>
@@ -862,15 +877,17 @@
         <v>15</v>
       </c>
       <c r="O4" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="P4" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="P4" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q4" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="Q4" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="R4" s="2"/>
+      <c r="R4" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
@@ -878,8 +895,9 @@
       <c r="W4" s="2"/>
       <c r="X4" s="2"/>
       <c r="Y4" s="2"/>
-    </row>
-    <row r="5" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="Z4" s="2"/>
+    </row>
+    <row r="5" spans="1:26" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="10" t="s">
         <v>7</v>
@@ -921,15 +939,17 @@
         <v>15</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="P5" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="Q5" s="13" t="s">
+      <c r="R5" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="R5" s="2"/>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
@@ -937,8 +957,9 @@
       <c r="W5" s="2"/>
       <c r="X5" s="2"/>
       <c r="Y5" s="2"/>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z5" s="2"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="3"/>
@@ -955,8 +976,8 @@
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="2"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="4"/>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
@@ -964,8 +985,9 @@
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
       <c r="Y6" s="2"/>
-    </row>
-    <row r="7" spans="1:25" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="Z6" s="2"/>
+    </row>
+    <row r="7" spans="1:26" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="5"/>
@@ -986,10 +1008,10 @@
       <c r="N7" s="14"/>
       <c r="O7" s="14"/>
       <c r="P7" s="14"/>
-      <c r="Q7" s="15" t="s">
+      <c r="Q7" s="14"/>
+      <c r="R7" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="R7" s="2"/>
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
@@ -997,8 +1019,9 @@
       <c r="W7" s="2"/>
       <c r="X7" s="2"/>
       <c r="Y7" s="2"/>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z7" s="2"/>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="5"/>
@@ -1015,10 +1038,12 @@
       <c r="L8" s="14"/>
       <c r="M8" s="14"/>
       <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
+      <c r="O8" s="14" t="s">
+        <v>54</v>
+      </c>
       <c r="P8" s="14"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="2"/>
+      <c r="Q8" s="14"/>
+      <c r="R8" s="16"/>
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
@@ -1026,8 +1051,9 @@
       <c r="W8" s="2"/>
       <c r="X8" s="2"/>
       <c r="Y8" s="2"/>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z8" s="2"/>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="5"/>
@@ -1046,8 +1072,8 @@
       <c r="N9" s="14"/>
       <c r="O9" s="14"/>
       <c r="P9" s="14"/>
-      <c r="Q9" s="16"/>
-      <c r="R9" s="2"/>
+      <c r="Q9" s="14"/>
+      <c r="R9" s="16"/>
       <c r="S9" s="2"/>
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
@@ -1055,8 +1081,9 @@
       <c r="W9" s="2"/>
       <c r="X9" s="2"/>
       <c r="Y9" s="2"/>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z9" s="2"/>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="5"/>
@@ -1075,8 +1102,8 @@
       <c r="N10" s="14"/>
       <c r="O10" s="14"/>
       <c r="P10" s="14"/>
-      <c r="Q10" s="16"/>
-      <c r="R10" s="2"/>
+      <c r="Q10" s="14"/>
+      <c r="R10" s="16"/>
       <c r="S10" s="2"/>
       <c r="T10" s="2"/>
       <c r="U10" s="2"/>
@@ -1084,8 +1111,9 @@
       <c r="W10" s="2"/>
       <c r="X10" s="2"/>
       <c r="Y10" s="2"/>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z10" s="2"/>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="5"/>
@@ -1104,8 +1132,8 @@
       <c r="N11" s="14"/>
       <c r="O11" s="14"/>
       <c r="P11" s="14"/>
-      <c r="Q11" s="16"/>
-      <c r="R11" s="2"/>
+      <c r="Q11" s="14"/>
+      <c r="R11" s="16"/>
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
@@ -1113,8 +1141,9 @@
       <c r="W11" s="2"/>
       <c r="X11" s="2"/>
       <c r="Y11" s="2"/>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z11" s="2"/>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="5"/>
@@ -1131,7 +1160,7 @@
       <c r="N12" s="5"/>
       <c r="O12" s="5"/>
       <c r="P12" s="5"/>
-      <c r="Q12" s="2"/>
+      <c r="Q12" s="5"/>
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
@@ -1140,8 +1169,9 @@
       <c r="W12" s="2"/>
       <c r="X12" s="2"/>
       <c r="Y12" s="2"/>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z12" s="2"/>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="5"/>
@@ -1158,7 +1188,7 @@
       <c r="N13" s="5"/>
       <c r="O13" s="5"/>
       <c r="P13" s="5"/>
-      <c r="Q13" s="2"/>
+      <c r="Q13" s="5"/>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
@@ -1167,8 +1197,9 @@
       <c r="W13" s="2"/>
       <c r="X13" s="2"/>
       <c r="Y13" s="2"/>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z13" s="2"/>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="5"/>
@@ -1185,7 +1216,7 @@
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
       <c r="P14" s="5"/>
-      <c r="Q14" s="2"/>
+      <c r="Q14" s="5"/>
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
@@ -1194,8 +1225,9 @@
       <c r="W14" s="2"/>
       <c r="X14" s="2"/>
       <c r="Y14" s="2"/>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z14" s="2"/>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="5"/>
@@ -1212,7 +1244,7 @@
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
       <c r="P15" s="5"/>
-      <c r="Q15" s="2"/>
+      <c r="Q15" s="5"/>
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
       <c r="T15" s="2"/>
@@ -1221,8 +1253,9 @@
       <c r="W15" s="2"/>
       <c r="X15" s="2"/>
       <c r="Y15" s="2"/>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z15" s="2"/>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="5"/>
@@ -1239,7 +1272,7 @@
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
       <c r="P16" s="5"/>
-      <c r="Q16" s="2"/>
+      <c r="Q16" s="5"/>
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
@@ -1248,8 +1281,9 @@
       <c r="W16" s="2"/>
       <c r="X16" s="2"/>
       <c r="Y16" s="2"/>
-    </row>
-    <row r="17" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="Z16" s="2"/>
+    </row>
+    <row r="17" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B17" s="2"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -1265,7 +1299,7 @@
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
       <c r="P17" s="5"/>
-      <c r="Q17" s="2"/>
+      <c r="Q17" s="5"/>
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
@@ -1274,8 +1308,9 @@
       <c r="W17" s="2"/>
       <c r="X17" s="2"/>
       <c r="Y17" s="2"/>
-    </row>
-    <row r="18" spans="2:25" x14ac:dyDescent="0.3">
+      <c r="Z17" s="2"/>
+    </row>
+    <row r="18" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B18" s="2"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -1291,7 +1326,7 @@
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
       <c r="P18" s="5"/>
-      <c r="Q18" s="2"/>
+      <c r="Q18" s="5"/>
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
@@ -1300,6 +1335,7 @@
       <c r="W18" s="2"/>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
+      <c r="Z18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>